<commit_message>
finetuning datavalidity script in template
</commit_message>
<xml_diff>
--- a/inst/templates/DataImportConfiguration.xlsx
+++ b/inst/templates/DataImportConfiguration.xlsx
@@ -14,16 +14,15 @@
     <sheet name="_Validity" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="validity_DataFiles_DataClass_5">'_Validity'!$A$2:$A$6</definedName>
-    <definedName name="validity_tpDictionary_Type_7">'_Validity'!$A$8:$A$12</definedName>
-    <definedName name="validity_pkDictionary_Type_14">'_Validity'!$A$14:$A$18</definedName>
+    <definedName name="validity_dataclassValues">'_Validity'!$A$1:$A$5</definedName>
+    <definedName name="validity_dictionaryTypeValues">'_Validity'!$A$7:$A$11</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="152">
   <si>
     <t xml:space="preserve">FileIdentifier</t>
   </si>
@@ -467,6 +466,18 @@
   </si>
   <si>
     <t xml:space="preserve">numericValues</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tp Aggregated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pk Individual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pk Aggregated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">numeric Values</t>
   </si>
 </sst>
 </file>
@@ -3959,6 +3970,56 @@
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_DataFiles_DataClass_5</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_DataFiles_DataClass_5</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_DataFiles_DataClass_5</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_DataFiles_DataClass_5</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_dataclassValues</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
   </extLst>
 </worksheet>
 </file>
@@ -4568,6 +4629,56 @@
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_tpDictionary_Type_7</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_tpDictionary_Type_7</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_tpDictionary_Type_7</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_tpDictionary_Type_7</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_dictionaryTypeValues</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
   </extLst>
 </worksheet>
 </file>
@@ -5143,6 +5254,56 @@
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_pkDictionary_Type_14</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_pkDictionary_Type_14</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_pkDictionary_Type_14</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_pkDictionary_Type_14</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>validity_dictionaryTypeValues</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
   </extLst>
 </worksheet>
 </file>
@@ -5248,81 +5409,51 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>142</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>147</v>
+        <v>151</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>